<commit_message>
Fix encoding bugs, update README, fix PostgreSQL upsert logic
</commit_message>
<xml_diff>
--- a/data/exports/AQI_India_Report.xlsx
+++ b/data/exports/AQI_India_Report.xlsx
@@ -7,9 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="All Cities" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Most Polluted" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Category Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="AQI Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -446,12 +445,12 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>air_quality_label</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>timestamp</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>air_quality_label</t>
         </is>
       </c>
     </row>
@@ -462,25 +461,25 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C2" t="n">
-        <v>44</v>
+        <v>42.5</v>
       </c>
       <c r="D2" t="n">
-        <v>51.6</v>
+        <v>49.1</v>
       </c>
       <c r="E2" t="n">
-        <v>547</v>
+        <v>681</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>29-05-2026 11:14</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>2026-05-29 17:52:42</t>
         </is>
       </c>
     </row>
@@ -491,25 +490,25 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="C3" t="n">
-        <v>9.699999999999999</v>
+        <v>18.9</v>
       </c>
       <c r="D3" t="n">
-        <v>12.1</v>
+        <v>24.7</v>
       </c>
       <c r="E3" t="n">
-        <v>400</v>
+        <v>680</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>29-05-2026 11:14</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>2026-05-29 17:52:43</t>
         </is>
       </c>
     </row>
@@ -520,25 +519,25 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C4" t="n">
-        <v>20.1</v>
+        <v>20.5</v>
       </c>
       <c r="D4" t="n">
-        <v>38.3</v>
+        <v>40.3</v>
       </c>
       <c r="E4" t="n">
-        <v>170</v>
+        <v>186</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>29-05-2026 11:14</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>2026-05-29 17:52:44</t>
         </is>
       </c>
     </row>
@@ -549,25 +548,25 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="C5" t="n">
-        <v>9.1</v>
+        <v>13</v>
       </c>
       <c r="D5" t="n">
-        <v>14.1</v>
+        <v>20.5</v>
       </c>
       <c r="E5" t="n">
-        <v>148</v>
+        <v>166</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>29-05-2026 11:14</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>2026-05-29 17:52:44</t>
         </is>
       </c>
     </row>
@@ -578,25 +577,25 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>327</v>
+        <v>277</v>
       </c>
       <c r="C6" t="n">
-        <v>110.6</v>
+        <v>105.7</v>
       </c>
       <c r="D6" t="n">
-        <v>555.1</v>
+        <v>551.3</v>
       </c>
       <c r="E6" t="n">
-        <v>427</v>
+        <v>550</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>29-05-2026 11:14</t>
+          <t>Hazardous</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Hazardous</t>
+          <t>2026-05-29 17:52:45</t>
         </is>
       </c>
     </row>
@@ -607,25 +606,25 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C7" t="n">
-        <v>20.3</v>
+        <v>25.9</v>
       </c>
       <c r="D7" t="n">
-        <v>23.3</v>
+        <v>34.3</v>
       </c>
       <c r="E7" t="n">
-        <v>376</v>
+        <v>315</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>29-05-2026 11:14</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>2026-05-29 17:52:46</t>
         </is>
       </c>
     </row>
@@ -636,25 +635,25 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C8" t="n">
-        <v>33.2</v>
+        <v>36.1</v>
       </c>
       <c r="D8" t="n">
-        <v>55.3</v>
+        <v>55.1</v>
       </c>
       <c r="E8" t="n">
-        <v>344</v>
+        <v>524</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>29-05-2026 11:14</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>2026-05-29 17:52:47</t>
         </is>
       </c>
     </row>
@@ -665,25 +664,25 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="C9" t="n">
-        <v>11</v>
+        <v>11.1</v>
       </c>
       <c r="D9" t="n">
-        <v>12.7</v>
+        <v>14.4</v>
       </c>
       <c r="E9" t="n">
-        <v>272</v>
+        <v>300</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>29-05-2026 11:14</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>2026-05-29 17:52:48</t>
         </is>
       </c>
     </row>
@@ -694,25 +693,25 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="C10" t="n">
-        <v>23.1</v>
+        <v>24</v>
       </c>
       <c r="D10" t="n">
-        <v>51.3</v>
+        <v>55.5</v>
       </c>
       <c r="E10" t="n">
-        <v>139</v>
+        <v>151</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>29-05-2026 11:14</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>2026-05-29 17:52:49</t>
         </is>
       </c>
     </row>
@@ -723,25 +722,25 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="C11" t="n">
-        <v>43.8</v>
+        <v>44</v>
       </c>
       <c r="D11" t="n">
-        <v>209.5</v>
+        <v>207.2</v>
       </c>
       <c r="E11" t="n">
-        <v>188</v>
+        <v>227</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>29-05-2026 11:14</t>
+          <t>Unhealthy</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Unhealthy</t>
+          <t>2026-05-29 17:52:49</t>
         </is>
       </c>
     </row>
@@ -752,25 +751,25 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C12" t="n">
-        <v>36.4</v>
+        <v>35</v>
       </c>
       <c r="D12" t="n">
-        <v>56.1</v>
+        <v>61.9</v>
       </c>
       <c r="E12" t="n">
-        <v>362</v>
+        <v>335</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>29-05-2026 11:14</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>2026-05-29 17:52:50</t>
         </is>
       </c>
     </row>
@@ -784,22 +783,22 @@
         <v>43</v>
       </c>
       <c r="C13" t="n">
-        <v>26.8</v>
+        <v>25.3</v>
       </c>
       <c r="D13" t="n">
-        <v>51.6</v>
+        <v>54.7</v>
       </c>
       <c r="E13" t="n">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>29-05-2026 11:14</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>2026-05-29 17:52:51</t>
         </is>
       </c>
     </row>
@@ -810,25 +809,25 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>63</v>
+        <v>46</v>
       </c>
       <c r="C14" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="D14" t="n">
-        <v>41</v>
+        <v>32.8</v>
       </c>
       <c r="E14" t="n">
-        <v>175</v>
+        <v>160</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>29-05-2026 11:14</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>2026-05-29 17:52:52</t>
         </is>
       </c>
     </row>
@@ -839,25 +838,25 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C15" t="n">
-        <v>32.2</v>
+        <v>27.1</v>
       </c>
       <c r="D15" t="n">
-        <v>43.5</v>
+        <v>33.9</v>
       </c>
       <c r="E15" t="n">
-        <v>299</v>
+        <v>320</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>29-05-2026 11:14</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>2026-05-29 17:52:53</t>
         </is>
       </c>
     </row>
@@ -868,25 +867,25 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="C16" t="n">
-        <v>27.3</v>
+        <v>27.1</v>
       </c>
       <c r="D16" t="n">
-        <v>58.8</v>
+        <v>55.9</v>
       </c>
       <c r="E16" t="n">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>29-05-2026 11:14</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>2026-05-29 17:52:54</t>
         </is>
       </c>
     </row>
@@ -897,25 +896,25 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C17" t="n">
-        <v>26.1</v>
+        <v>27.2</v>
       </c>
       <c r="D17" t="n">
-        <v>58.2</v>
+        <v>53.7</v>
       </c>
       <c r="E17" t="n">
-        <v>219</v>
+        <v>179</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>29-05-2026 11:14</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>2026-05-29 17:52:55</t>
         </is>
       </c>
     </row>
@@ -926,25 +925,25 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C18" t="n">
-        <v>4.1</v>
+        <v>3.1</v>
       </c>
       <c r="D18" t="n">
-        <v>6</v>
+        <v>3.7</v>
       </c>
       <c r="E18" t="n">
         <v>159</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>29-05-2026 11:14</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>2026-05-29 17:52:56</t>
         </is>
       </c>
     </row>
@@ -955,25 +954,25 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="C19" t="n">
-        <v>6.4</v>
+        <v>4.8</v>
       </c>
       <c r="D19" t="n">
-        <v>7.7</v>
+        <v>6.5</v>
       </c>
       <c r="E19" t="n">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>29-05-2026 11:14</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>2026-05-29 17:52:56</t>
         </is>
       </c>
     </row>
@@ -984,25 +983,25 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C20" t="n">
-        <v>36.7</v>
+        <v>35.5</v>
       </c>
       <c r="D20" t="n">
-        <v>114.6</v>
+        <v>111.1</v>
       </c>
       <c r="E20" t="n">
-        <v>334</v>
+        <v>476</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>29-05-2026 11:14</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>2026-05-29 17:52:57</t>
         </is>
       </c>
     </row>
@@ -1016,22 +1015,22 @@
         <v>73</v>
       </c>
       <c r="C21" t="n">
-        <v>45.5</v>
+        <v>40.5</v>
       </c>
       <c r="D21" t="n">
-        <v>53.8</v>
+        <v>61</v>
       </c>
       <c r="E21" t="n">
-        <v>426</v>
+        <v>458</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>29-05-2026 11:14</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>2026-05-29 17:52:58</t>
         </is>
       </c>
     </row>
@@ -1042,25 +1041,25 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>506</v>
+        <v>408</v>
       </c>
       <c r="C22" t="n">
-        <v>339.9</v>
+        <v>143.4</v>
       </c>
       <c r="D22" t="n">
-        <v>2801.4</v>
+        <v>1154.8</v>
       </c>
       <c r="E22" t="n">
-        <v>381</v>
+        <v>242</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>29-05-2026 11:14</t>
+          <t>Hazardous</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Hazardous</t>
+          <t>2026-05-29 17:52:59</t>
         </is>
       </c>
     </row>
@@ -1071,25 +1070,25 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="C23" t="n">
-        <v>32.1</v>
+        <v>39.9</v>
       </c>
       <c r="D23" t="n">
-        <v>53.9</v>
+        <v>50.8</v>
       </c>
       <c r="E23" t="n">
-        <v>273</v>
+        <v>671</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>29-05-2026 11:14</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>2026-05-29 17:53:00</t>
         </is>
       </c>
     </row>
@@ -1100,25 +1099,25 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="C24" t="n">
-        <v>5.8</v>
+        <v>7.2</v>
       </c>
       <c r="D24" t="n">
-        <v>7.5</v>
+        <v>9.4</v>
       </c>
       <c r="E24" t="n">
-        <v>144</v>
+        <v>198</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>29-05-2026 11:14</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>2026-05-29 17:53:01</t>
         </is>
       </c>
     </row>
@@ -1129,25 +1128,25 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C25" t="n">
-        <v>36</v>
+        <v>38.1</v>
       </c>
       <c r="D25" t="n">
-        <v>56.2</v>
+        <v>55.5</v>
       </c>
       <c r="E25" t="n">
-        <v>320</v>
+        <v>463</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>29-05-2026 11:14</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>2026-05-29 17:53:02</t>
         </is>
       </c>
     </row>
@@ -1158,25 +1157,25 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C26" t="n">
-        <v>38.5</v>
+        <v>36.6</v>
       </c>
       <c r="D26" t="n">
-        <v>50.1</v>
+        <v>45.9</v>
       </c>
       <c r="E26" t="n">
-        <v>267</v>
+        <v>430</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>29-05-2026 11:14</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>2026-05-29 17:53:02</t>
         </is>
       </c>
     </row>
@@ -1191,274 +1190,59 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>city</t>
+          <t>Air Quality Label</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>aqi_index</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>air_quality_label</t>
+          <t>City Count</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Agra</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>506</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Hazardous</t>
-        </is>
+        <v>9</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Delhi</t>
+          <t>Hazardous</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>327</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Hazardous</t>
-        </is>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Jaipur</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>117</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Unhealthy</t>
-        </is>
+        <v>13</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Visakhapatnam</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>75</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Chandigarh</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>75</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Varanasi</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>73</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Guwahati</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>73</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Kolkata</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>70</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Patna</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>70</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Ranchi</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>70</v>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>air_quality_label</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>total_cities</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>avg_aqi</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>max_aqi</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Good</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>8</v>
-      </c>
-      <c r="C2" t="n">
-        <v>36.5</v>
-      </c>
-      <c r="D2" t="n">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Hazardous</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>2</v>
-      </c>
-      <c r="C3" t="n">
-        <v>416.5</v>
-      </c>
-      <c r="D3" t="n">
-        <v>506</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>14</v>
-      </c>
-      <c r="C4" t="n">
-        <v>67.06999999999999</v>
-      </c>
-      <c r="D4" t="n">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
           <t>Unhealthy</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>1</v>
-      </c>
-      <c r="C5" t="n">
-        <v>117</v>
-      </c>
-      <c r="D5" t="n">
-        <v>117</v>
       </c>
     </row>
   </sheetData>

</xml_diff>